<commit_message>
update formualas functionality in generate_assigment_report.py
</commit_message>
<xml_diff>
--- a/Assignment_Deliverable.xlsx
+++ b/Assignment_Deliverable.xlsx
@@ -415,58 +415,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Methodology &amp; Justification</t>
+          <t>Industry Choice: Fast-Moving Consumer Goods (FMCG) via Quick Commerce.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Industry Choice: Fast-Moving Consumer Goods (FMCG) via Quick Commerce.</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Justification: Highly standardized SKUs allowing for true apples-to-apples comparison, high-frequency algorithmic pricing updates, and high relevance to real-world household expenditure inflation.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Justification: Highly standardized SKUs allowing for true apples-to-apples comparison, high-frequency algorithmic pricing updates, and high relevance to real-world household expenditure inflation.</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fields Scraped: Timestamp, SKU ID, Active Listed Pack Size, Current Selling Price, and Availability Status. MRP is omitted as continuous promotions make transaction price the true market clearer.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Fields Scraped: Timestamp, SKU ID, Active Listed Pack Size, Current Selling Price, and Availability Status. MRP is omitted as continuous promotions make transaction price the true market clearer.</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Handling Stockouts: Implemented a Carry-Forward imputation model. If an item is out of stock (e.g., Eggs on Day 4), the script carries forward the last observed normalized price from the prior day to maintain index continuity.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Handling Stockouts: Implemented a Carry-Forward imputation model. If an item is out of stock (e.g., Eggs on Day 4), the script carries forward the last observed normalized price from the prior day to maintain index continuity.</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Handling Shrinkflation: Developed a pre-averaging mathematical normalization engine. The scraper extracts the active pack size from the page DOM and normalizes the selling price to a base unit (Price per 100g or Price per 1 unit) before averaging, ensuring the index tracks pure inflation, not packaging changes.</t>
         </is>
@@ -524,12 +517,12 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Base_Price</t>
+          <t>Base Price</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Price_Relative</t>
+          <t>Price Relative</t>
         </is>
       </c>
     </row>
@@ -563,11 +556,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H2" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="I2" t="n">
-        <v>100</v>
+      <c r="H2">
+        <f>XLOOKUP(C2, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>(F2/H2)*100</f>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -600,11 +595,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H3" t="n">
-        <v>57</v>
-      </c>
-      <c r="I3" t="n">
-        <v>100</v>
+      <c r="H3">
+        <f>XLOOKUP(C3, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I3">
+        <f>(F3/H3)*100</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -637,11 +634,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H4" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="I4" t="n">
-        <v>100</v>
+      <c r="H4">
+        <f>XLOOKUP(C4, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I4">
+        <f>(F4/H4)*100</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -674,11 +673,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H5" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="I5" t="n">
-        <v>100</v>
+      <c r="H5">
+        <f>XLOOKUP(C5, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I5">
+        <f>(F5/H5)*100</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -711,11 +712,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H6" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="I6" t="n">
-        <v>100</v>
+      <c r="H6">
+        <f>XLOOKUP(C6, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I6">
+        <f>(F6/H6)*100</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -748,11 +751,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H7" t="n">
-        <v>86.67</v>
-      </c>
-      <c r="I7" t="n">
-        <v>100</v>
+      <c r="H7">
+        <f>XLOOKUP(C7, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I7">
+        <f>(F7/H7)*100</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -785,11 +790,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H8" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="I8" t="n">
-        <v>100</v>
+      <c r="H8">
+        <f>XLOOKUP(C8, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>(F8/H8)*100</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -822,11 +829,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H9" t="n">
-        <v>18.57</v>
-      </c>
-      <c r="I9" t="n">
-        <v>100</v>
+      <c r="H9">
+        <f>XLOOKUP(C9, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I9">
+        <f>(F9/H9)*100</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -859,11 +868,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H10" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="I10" t="n">
-        <v>100</v>
+      <c r="H10">
+        <f>XLOOKUP(C10, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I10">
+        <f>(F10/H10)*100</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -896,11 +907,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H11" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="I11" t="n">
-        <v>100</v>
+      <c r="H11">
+        <f>XLOOKUP(C11, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I11">
+        <f>(F11/H11)*100</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -933,11 +946,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H12" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="I12" t="n">
-        <v>100</v>
+      <c r="H12">
+        <f>XLOOKUP(C12, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I12">
+        <f>(F12/H12)*100</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -970,11 +985,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H13" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="I13" t="n">
-        <v>100</v>
+      <c r="H13">
+        <f>XLOOKUP(C13, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I13">
+        <f>(F13/H13)*100</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1007,11 +1024,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H14" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="I14" t="n">
-        <v>100</v>
+      <c r="H14">
+        <f>XLOOKUP(C14, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I14">
+        <f>(F14/H14)*100</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -1044,11 +1063,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H15" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="I15" t="n">
-        <v>100</v>
+      <c r="H15">
+        <f>XLOOKUP(C15, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I15">
+        <f>(F15/H15)*100</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -1081,11 +1102,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H16" t="n">
-        <v>446</v>
-      </c>
-      <c r="I16" t="n">
-        <v>100</v>
+      <c r="H16">
+        <f>XLOOKUP(C16, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I16">
+        <f>(F16/H16)*100</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -1118,11 +1141,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H17" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="I17" t="n">
-        <v>100</v>
+      <c r="H17">
+        <f>XLOOKUP(C17, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I17">
+        <f>(F17/H17)*100</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -1155,11 +1180,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H18" t="n">
-        <v>6.12</v>
-      </c>
-      <c r="I18" t="n">
-        <v>100</v>
+      <c r="H18">
+        <f>XLOOKUP(C18, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I18">
+        <f>(F18/H18)*100</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1192,11 +1219,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H19" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="I19" t="n">
-        <v>100</v>
+      <c r="H19">
+        <f>XLOOKUP(C19, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I19">
+        <f>(F19/H19)*100</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1229,11 +1258,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H20" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="I20" t="n">
-        <v>100</v>
+      <c r="H20">
+        <f>XLOOKUP(C20, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I20">
+        <f>(F20/H20)*100</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1266,11 +1297,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H21" t="n">
-        <v>6</v>
-      </c>
-      <c r="I21" t="n">
-        <v>100</v>
+      <c r="H21">
+        <f>XLOOKUP(C21, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I21">
+        <f>(F21/H21)*100</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1303,11 +1336,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H22" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="I22" t="n">
-        <v>100</v>
+      <c r="H22">
+        <f>XLOOKUP(C22, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I22">
+        <f>(F22/H22)*100</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -1340,11 +1375,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H23" t="n">
-        <v>57</v>
-      </c>
-      <c r="I23" t="n">
-        <v>100</v>
+      <c r="H23">
+        <f>XLOOKUP(C23, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I23">
+        <f>(F23/H23)*100</f>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -1377,11 +1414,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H24" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="I24" t="n">
-        <v>100.8771929824561</v>
+      <c r="H24">
+        <f>XLOOKUP(C24, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I24">
+        <f>(F24/H24)*100</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1414,11 +1453,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H25" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="I25" t="n">
-        <v>100</v>
+      <c r="H25">
+        <f>XLOOKUP(C25, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I25">
+        <f>(F25/H25)*100</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1451,11 +1492,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H26" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="I26" t="n">
-        <v>100</v>
+      <c r="H26">
+        <f>XLOOKUP(C26, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I26">
+        <f>(F26/H26)*100</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1488,11 +1531,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H27" t="n">
-        <v>86.67</v>
-      </c>
-      <c r="I27" t="n">
-        <v>100</v>
+      <c r="H27">
+        <f>XLOOKUP(C27, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I27">
+        <f>(F27/H27)*100</f>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1525,11 +1570,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H28" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="I28" t="n">
-        <v>100</v>
+      <c r="H28">
+        <f>XLOOKUP(C28, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I28">
+        <f>(F28/H28)*100</f>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -1562,11 +1609,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H29" t="n">
-        <v>18.57</v>
-      </c>
-      <c r="I29" t="n">
-        <v>100</v>
+      <c r="H29">
+        <f>XLOOKUP(C29, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I29">
+        <f>(F29/H29)*100</f>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1599,11 +1648,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H30" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="I30" t="n">
-        <v>100</v>
+      <c r="H30">
+        <f>XLOOKUP(C30, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I30">
+        <f>(F30/H30)*100</f>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -1636,11 +1687,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H31" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="I31" t="n">
-        <v>104.8780487804878</v>
+      <c r="H31">
+        <f>XLOOKUP(C31, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I31">
+        <f>(F31/H31)*100</f>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -1673,11 +1726,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="I32" t="n">
-        <v>100</v>
+      <c r="H32">
+        <f>XLOOKUP(C32, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I32">
+        <f>(F32/H32)*100</f>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -1710,11 +1765,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H33" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="I33" t="n">
-        <v>109.2592592592593</v>
+      <c r="H33">
+        <f>XLOOKUP(C33, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I33">
+        <f>(F33/H33)*100</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -1747,11 +1804,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H34" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="I34" t="n">
-        <v>100</v>
+      <c r="H34">
+        <f>XLOOKUP(C34, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I34">
+        <f>(F34/H34)*100</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -1784,11 +1843,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H35" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="I35" t="n">
-        <v>100</v>
+      <c r="H35">
+        <f>XLOOKUP(C35, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I35">
+        <f>(F35/H35)*100</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -1821,11 +1882,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H36" t="n">
-        <v>446</v>
-      </c>
-      <c r="I36" t="n">
-        <v>100</v>
+      <c r="H36">
+        <f>XLOOKUP(C36, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I36">
+        <f>(F36/H36)*100</f>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -1858,11 +1921,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H37" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="I37" t="n">
-        <v>100</v>
+      <c r="H37">
+        <f>XLOOKUP(C37, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I37">
+        <f>(F37/H37)*100</f>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -1895,11 +1960,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H38" t="n">
-        <v>6.12</v>
-      </c>
-      <c r="I38" t="n">
-        <v>100</v>
+      <c r="H38">
+        <f>XLOOKUP(C38, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I38">
+        <f>(F38/H38)*100</f>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -1932,11 +1999,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H39" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="I39" t="n">
-        <v>100</v>
+      <c r="H39">
+        <f>XLOOKUP(C39, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I39">
+        <f>(F39/H39)*100</f>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -1969,11 +2038,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H40" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="I40" t="n">
-        <v>100</v>
+      <c r="H40">
+        <f>XLOOKUP(C40, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I40">
+        <f>(F40/H40)*100</f>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -2006,11 +2077,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H41" t="n">
-        <v>6</v>
-      </c>
-      <c r="I41" t="n">
-        <v>100</v>
+      <c r="H41">
+        <f>XLOOKUP(C41, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I41">
+        <f>(F41/H41)*100</f>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -2043,11 +2116,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H42" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="I42" t="n">
-        <v>100</v>
+      <c r="H42">
+        <f>XLOOKUP(C42, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I42">
+        <f>(F42/H42)*100</f>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -2080,11 +2155,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H43" t="n">
-        <v>57</v>
-      </c>
-      <c r="I43" t="n">
-        <v>100</v>
+      <c r="H43">
+        <f>XLOOKUP(C43, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I43">
+        <f>(F43/H43)*100</f>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -2117,11 +2194,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H44" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="I44" t="n">
-        <v>103.5087719298246</v>
+      <c r="H44">
+        <f>XLOOKUP(C44, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I44">
+        <f>(F44/H44)*100</f>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -2154,11 +2233,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H45" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="I45" t="n">
-        <v>101.123595505618</v>
+      <c r="H45">
+        <f>XLOOKUP(C45, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I45">
+        <f>(F45/H45)*100</f>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -2191,11 +2272,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H46" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="I46" t="n">
-        <v>100</v>
+      <c r="H46">
+        <f>XLOOKUP(C46, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I46">
+        <f>(F46/H46)*100</f>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -2228,11 +2311,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H47" t="n">
-        <v>86.67</v>
-      </c>
-      <c r="I47" t="n">
-        <v>100</v>
+      <c r="H47">
+        <f>XLOOKUP(C47, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I47">
+        <f>(F47/H47)*100</f>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -2265,11 +2350,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H48" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="I48" t="n">
-        <v>100</v>
+      <c r="H48">
+        <f>XLOOKUP(C48, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I48">
+        <f>(F48/H48)*100</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -2302,11 +2389,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H49" t="n">
-        <v>18.57</v>
-      </c>
-      <c r="I49" t="n">
-        <v>101.2385568120625</v>
+      <c r="H49">
+        <f>XLOOKUP(C49, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I49">
+        <f>(F49/H49)*100</f>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -2339,11 +2428,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H50" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="I50" t="n">
-        <v>100</v>
+      <c r="H50">
+        <f>XLOOKUP(C50, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I50">
+        <f>(F50/H50)*100</f>
+        <v/>
       </c>
     </row>
     <row r="51">
@@ -2376,11 +2467,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H51" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="I51" t="n">
-        <v>112.1951219512195</v>
+      <c r="H51">
+        <f>XLOOKUP(C51, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I51">
+        <f>(F51/H51)*100</f>
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -2413,11 +2506,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H52" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="I52" t="n">
-        <v>105.5555555555556</v>
+      <c r="H52">
+        <f>XLOOKUP(C52, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I52">
+        <f>(F52/H52)*100</f>
+        <v/>
       </c>
     </row>
     <row r="53">
@@ -2450,11 +2545,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H53" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="I53" t="n">
-        <v>120.3703703703704</v>
+      <c r="H53">
+        <f>XLOOKUP(C53, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I53">
+        <f>(F53/H53)*100</f>
+        <v/>
       </c>
     </row>
     <row r="54">
@@ -2487,11 +2584,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H54" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="I54" t="n">
-        <v>102.0408163265306</v>
+      <c r="H54">
+        <f>XLOOKUP(C54, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I54">
+        <f>(F54/H54)*100</f>
+        <v/>
       </c>
     </row>
     <row r="55">
@@ -2524,11 +2623,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H55" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="I55" t="n">
-        <v>100</v>
+      <c r="H55">
+        <f>XLOOKUP(C55, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I55">
+        <f>(F55/H55)*100</f>
+        <v/>
       </c>
     </row>
     <row r="56">
@@ -2561,11 +2662,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H56" t="n">
-        <v>446</v>
-      </c>
-      <c r="I56" t="n">
-        <v>100</v>
+      <c r="H56">
+        <f>XLOOKUP(C56, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I56">
+        <f>(F56/H56)*100</f>
+        <v/>
       </c>
     </row>
     <row r="57">
@@ -2598,11 +2701,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H57" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="I57" t="n">
-        <v>100</v>
+      <c r="H57">
+        <f>XLOOKUP(C57, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I57">
+        <f>(F57/H57)*100</f>
+        <v/>
       </c>
     </row>
     <row r="58">
@@ -2635,11 +2740,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H58" t="n">
-        <v>6.12</v>
-      </c>
-      <c r="I58" t="n">
-        <v>100.4901960784314</v>
+      <c r="H58">
+        <f>XLOOKUP(C58, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I58">
+        <f>(F58/H58)*100</f>
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -2672,11 +2779,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H59" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="I59" t="n">
-        <v>100</v>
+      <c r="H59">
+        <f>XLOOKUP(C59, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I59">
+        <f>(F59/H59)*100</f>
+        <v/>
       </c>
     </row>
     <row r="60">
@@ -2709,11 +2818,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H60" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="I60" t="n">
-        <v>100</v>
+      <c r="H60">
+        <f>XLOOKUP(C60, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I60">
+        <f>(F60/H60)*100</f>
+        <v/>
       </c>
     </row>
     <row r="61">
@@ -2746,11 +2857,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H61" t="n">
-        <v>6</v>
-      </c>
-      <c r="I61" t="n">
-        <v>100</v>
+      <c r="H61">
+        <f>XLOOKUP(C61, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I61">
+        <f>(F61/H61)*100</f>
+        <v/>
       </c>
     </row>
     <row r="62">
@@ -2783,11 +2896,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H62" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="I62" t="n">
-        <v>100</v>
+      <c r="H62">
+        <f>XLOOKUP(C62, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I62">
+        <f>(F62/H62)*100</f>
+        <v/>
       </c>
     </row>
     <row r="63">
@@ -2820,11 +2935,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H63" t="n">
-        <v>57</v>
-      </c>
-      <c r="I63" t="n">
-        <v>100</v>
+      <c r="H63">
+        <f>XLOOKUP(C63, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I63">
+        <f>(F63/H63)*100</f>
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -2857,11 +2974,13 @@
           <t>Imputed (Carry Forward)</t>
         </is>
       </c>
-      <c r="H64" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="I64" t="n">
-        <v>103.5087719298246</v>
+      <c r="H64">
+        <f>XLOOKUP(C64, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I64">
+        <f>(F64/H64)*100</f>
+        <v/>
       </c>
     </row>
     <row r="65">
@@ -2894,11 +3013,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H65" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="I65" t="n">
-        <v>101.123595505618</v>
+      <c r="H65">
+        <f>XLOOKUP(C65, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I65">
+        <f>(F65/H65)*100</f>
+        <v/>
       </c>
     </row>
     <row r="66">
@@ -2931,11 +3052,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H66" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="I66" t="n">
-        <v>100</v>
+      <c r="H66">
+        <f>XLOOKUP(C66, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I66">
+        <f>(F66/H66)*100</f>
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -2968,11 +3091,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H67" t="n">
-        <v>86.67</v>
-      </c>
-      <c r="I67" t="n">
-        <v>100</v>
+      <c r="H67">
+        <f>XLOOKUP(C67, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I67">
+        <f>(F67/H67)*100</f>
+        <v/>
       </c>
     </row>
     <row r="68">
@@ -3005,11 +3130,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H68" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="I68" t="n">
-        <v>100</v>
+      <c r="H68">
+        <f>XLOOKUP(C68, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I68">
+        <f>(F68/H68)*100</f>
+        <v/>
       </c>
     </row>
     <row r="69">
@@ -3042,11 +3169,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H69" t="n">
-        <v>18.57</v>
-      </c>
-      <c r="I69" t="n">
-        <v>101.2385568120625</v>
+      <c r="H69">
+        <f>XLOOKUP(C69, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I69">
+        <f>(F69/H69)*100</f>
+        <v/>
       </c>
     </row>
     <row r="70">
@@ -3079,11 +3208,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H70" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="I70" t="n">
-        <v>101.1904761904762</v>
+      <c r="H70">
+        <f>XLOOKUP(C70, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I70">
+        <f>(F70/H70)*100</f>
+        <v/>
       </c>
     </row>
     <row r="71">
@@ -3116,11 +3247,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H71" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="I71" t="n">
-        <v>117.0731707317073</v>
+      <c r="H71">
+        <f>XLOOKUP(C71, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I71">
+        <f>(F71/H71)*100</f>
+        <v/>
       </c>
     </row>
     <row r="72">
@@ -3153,11 +3286,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H72" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="I72" t="n">
-        <v>105.5555555555556</v>
+      <c r="H72">
+        <f>XLOOKUP(C72, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I72">
+        <f>(F72/H72)*100</f>
+        <v/>
       </c>
     </row>
     <row r="73">
@@ -3190,11 +3325,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H73" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="I73" t="n">
-        <v>125.9259259259259</v>
+      <c r="H73">
+        <f>XLOOKUP(C73, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I73">
+        <f>(F73/H73)*100</f>
+        <v/>
       </c>
     </row>
     <row r="74">
@@ -3227,11 +3364,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H74" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="I74" t="n">
-        <v>102.0408163265306</v>
+      <c r="H74">
+        <f>XLOOKUP(C74, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I74">
+        <f>(F74/H74)*100</f>
+        <v/>
       </c>
     </row>
     <row r="75">
@@ -3264,11 +3403,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H75" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="I75" t="n">
-        <v>100</v>
+      <c r="H75">
+        <f>XLOOKUP(C75, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I75">
+        <f>(F75/H75)*100</f>
+        <v/>
       </c>
     </row>
     <row r="76">
@@ -3301,11 +3442,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H76" t="n">
-        <v>446</v>
-      </c>
-      <c r="I76" t="n">
-        <v>100</v>
+      <c r="H76">
+        <f>XLOOKUP(C76, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I76">
+        <f>(F76/H76)*100</f>
+        <v/>
       </c>
     </row>
     <row r="77">
@@ -3338,11 +3481,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H77" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="I77" t="n">
-        <v>100</v>
+      <c r="H77">
+        <f>XLOOKUP(C77, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I77">
+        <f>(F77/H77)*100</f>
+        <v/>
       </c>
     </row>
     <row r="78">
@@ -3375,11 +3520,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H78" t="n">
-        <v>6.12</v>
-      </c>
-      <c r="I78" t="n">
-        <v>100.4901960784314</v>
+      <c r="H78">
+        <f>XLOOKUP(C78, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I78">
+        <f>(F78/H78)*100</f>
+        <v/>
       </c>
     </row>
     <row r="79">
@@ -3412,11 +3559,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H79" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="I79" t="n">
-        <v>100</v>
+      <c r="H79">
+        <f>XLOOKUP(C79, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I79">
+        <f>(F79/H79)*100</f>
+        <v/>
       </c>
     </row>
     <row r="80">
@@ -3449,11 +3598,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H80" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="I80" t="n">
-        <v>100</v>
+      <c r="H80">
+        <f>XLOOKUP(C80, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I80">
+        <f>(F80/H80)*100</f>
+        <v/>
       </c>
     </row>
     <row r="81">
@@ -3486,11 +3637,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H81" t="n">
-        <v>6</v>
-      </c>
-      <c r="I81" t="n">
-        <v>100</v>
+      <c r="H81">
+        <f>XLOOKUP(C81, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I81">
+        <f>(F81/H81)*100</f>
+        <v/>
       </c>
     </row>
     <row r="82">
@@ -3523,11 +3676,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H82" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="I82" t="n">
-        <v>100</v>
+      <c r="H82">
+        <f>XLOOKUP(C82, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I82">
+        <f>(F82/H82)*100</f>
+        <v/>
       </c>
     </row>
     <row r="83">
@@ -3560,11 +3715,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H83" t="n">
-        <v>57</v>
-      </c>
-      <c r="I83" t="n">
-        <v>100</v>
+      <c r="H83">
+        <f>XLOOKUP(C83, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I83">
+        <f>(F83/H83)*100</f>
+        <v/>
       </c>
     </row>
     <row r="84">
@@ -3597,11 +3754,13 @@
           <t>Imputed (Carry Forward)</t>
         </is>
       </c>
-      <c r="H84" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="I84" t="n">
-        <v>103.5087719298246</v>
+      <c r="H84">
+        <f>XLOOKUP(C84, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I84">
+        <f>(F84/H84)*100</f>
+        <v/>
       </c>
     </row>
     <row r="85">
@@ -3634,11 +3793,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H85" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="I85" t="n">
-        <v>101.123595505618</v>
+      <c r="H85">
+        <f>XLOOKUP(C85, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I85">
+        <f>(F85/H85)*100</f>
+        <v/>
       </c>
     </row>
     <row r="86">
@@ -3671,11 +3832,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H86" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="I86" t="n">
-        <v>100</v>
+      <c r="H86">
+        <f>XLOOKUP(C86, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I86">
+        <f>(F86/H86)*100</f>
+        <v/>
       </c>
     </row>
     <row r="87">
@@ -3708,11 +3871,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H87" t="n">
-        <v>86.67</v>
-      </c>
-      <c r="I87" t="n">
-        <v>100</v>
+      <c r="H87">
+        <f>XLOOKUP(C87, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I87">
+        <f>(F87/H87)*100</f>
+        <v/>
       </c>
     </row>
     <row r="88">
@@ -3745,11 +3910,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H88" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="I88" t="n">
-        <v>100</v>
+      <c r="H88">
+        <f>XLOOKUP(C88, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I88">
+        <f>(F88/H88)*100</f>
+        <v/>
       </c>
     </row>
     <row r="89">
@@ -3782,11 +3949,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H89" t="n">
-        <v>18.57</v>
-      </c>
-      <c r="I89" t="n">
-        <v>101.2385568120625</v>
+      <c r="H89">
+        <f>XLOOKUP(C89, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I89">
+        <f>(F89/H89)*100</f>
+        <v/>
       </c>
     </row>
     <row r="90">
@@ -3819,11 +3988,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H90" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="I90" t="n">
-        <v>101.1904761904762</v>
+      <c r="H90">
+        <f>XLOOKUP(C90, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I90">
+        <f>(F90/H90)*100</f>
+        <v/>
       </c>
     </row>
     <row r="91">
@@ -3856,11 +4027,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H91" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="I91" t="n">
-        <v>117.0731707317073</v>
+      <c r="H91">
+        <f>XLOOKUP(C91, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I91">
+        <f>(F91/H91)*100</f>
+        <v/>
       </c>
     </row>
     <row r="92">
@@ -3893,11 +4066,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H92" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="I92" t="n">
-        <v>108.3333333333333</v>
+      <c r="H92">
+        <f>XLOOKUP(C92, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I92">
+        <f>(F92/H92)*100</f>
+        <v/>
       </c>
     </row>
     <row r="93">
@@ -3930,11 +4105,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H93" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="I93" t="n">
-        <v>114.8148148148148</v>
+      <c r="H93">
+        <f>XLOOKUP(C93, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I93">
+        <f>(F93/H93)*100</f>
+        <v/>
       </c>
     </row>
     <row r="94">
@@ -3967,11 +4144,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H94" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="I94" t="n">
-        <v>102.0408163265306</v>
+      <c r="H94">
+        <f>XLOOKUP(C94, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I94">
+        <f>(F94/H94)*100</f>
+        <v/>
       </c>
     </row>
     <row r="95">
@@ -4004,11 +4183,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H95" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="I95" t="n">
-        <v>100</v>
+      <c r="H95">
+        <f>XLOOKUP(C95, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I95">
+        <f>(F95/H95)*100</f>
+        <v/>
       </c>
     </row>
     <row r="96">
@@ -4041,11 +4222,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H96" t="n">
-        <v>446</v>
-      </c>
-      <c r="I96" t="n">
-        <v>100</v>
+      <c r="H96">
+        <f>XLOOKUP(C96, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I96">
+        <f>(F96/H96)*100</f>
+        <v/>
       </c>
     </row>
     <row r="97">
@@ -4078,11 +4261,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H97" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="I97" t="n">
-        <v>100</v>
+      <c r="H97">
+        <f>XLOOKUP(C97, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I97">
+        <f>(F97/H97)*100</f>
+        <v/>
       </c>
     </row>
     <row r="98">
@@ -4115,11 +4300,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H98" t="n">
-        <v>6.12</v>
-      </c>
-      <c r="I98" t="n">
-        <v>100.4901960784314</v>
+      <c r="H98">
+        <f>XLOOKUP(C98, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I98">
+        <f>(F98/H98)*100</f>
+        <v/>
       </c>
     </row>
     <row r="99">
@@ -4152,11 +4339,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H99" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="I99" t="n">
-        <v>100</v>
+      <c r="H99">
+        <f>XLOOKUP(C99, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I99">
+        <f>(F99/H99)*100</f>
+        <v/>
       </c>
     </row>
     <row r="100">
@@ -4189,11 +4378,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H100" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="I100" t="n">
-        <v>100.5747126436782</v>
+      <c r="H100">
+        <f>XLOOKUP(C100, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I100">
+        <f>(F100/H100)*100</f>
+        <v/>
       </c>
     </row>
     <row r="101">
@@ -4226,11 +4417,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H101" t="n">
-        <v>6</v>
-      </c>
-      <c r="I101" t="n">
-        <v>100</v>
+      <c r="H101">
+        <f>XLOOKUP(C101, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I101">
+        <f>(F101/H101)*100</f>
+        <v/>
       </c>
     </row>
     <row r="102">
@@ -4263,11 +4456,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H102" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="I102" t="n">
-        <v>100</v>
+      <c r="H102">
+        <f>XLOOKUP(C102, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I102">
+        <f>(F102/H102)*100</f>
+        <v/>
       </c>
     </row>
     <row r="103">
@@ -4300,11 +4495,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H103" t="n">
-        <v>57</v>
-      </c>
-      <c r="I103" t="n">
-        <v>100</v>
+      <c r="H103">
+        <f>XLOOKUP(C103, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I103">
+        <f>(F103/H103)*100</f>
+        <v/>
       </c>
     </row>
     <row r="104">
@@ -4337,11 +4534,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H104" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="I104" t="n">
-        <v>105.2631578947368</v>
+      <c r="H104">
+        <f>XLOOKUP(C104, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I104">
+        <f>(F104/H104)*100</f>
+        <v/>
       </c>
     </row>
     <row r="105">
@@ -4374,11 +4573,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H105" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="I105" t="n">
-        <v>101.123595505618</v>
+      <c r="H105">
+        <f>XLOOKUP(C105, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I105">
+        <f>(F105/H105)*100</f>
+        <v/>
       </c>
     </row>
     <row r="106">
@@ -4411,11 +4612,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H106" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="I106" t="n">
-        <v>100</v>
+      <c r="H106">
+        <f>XLOOKUP(C106, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I106">
+        <f>(F106/H106)*100</f>
+        <v/>
       </c>
     </row>
     <row r="107">
@@ -4448,11 +4651,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H107" t="n">
-        <v>86.67</v>
-      </c>
-      <c r="I107" t="n">
-        <v>100</v>
+      <c r="H107">
+        <f>XLOOKUP(C107, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I107">
+        <f>(F107/H107)*100</f>
+        <v/>
       </c>
     </row>
     <row r="108">
@@ -4485,11 +4690,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H108" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="I108" t="n">
-        <v>100</v>
+      <c r="H108">
+        <f>XLOOKUP(C108, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I108">
+        <f>(F108/H108)*100</f>
+        <v/>
       </c>
     </row>
     <row r="109">
@@ -4522,11 +4729,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H109" t="n">
-        <v>18.57</v>
-      </c>
-      <c r="I109" t="n">
-        <v>101.2385568120625</v>
+      <c r="H109">
+        <f>XLOOKUP(C109, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I109">
+        <f>(F109/H109)*100</f>
+        <v/>
       </c>
     </row>
     <row r="110">
@@ -4559,11 +4768,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H110" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="I110" t="n">
-        <v>101.1904761904762</v>
+      <c r="H110">
+        <f>XLOOKUP(C110, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I110">
+        <f>(F110/H110)*100</f>
+        <v/>
       </c>
     </row>
     <row r="111">
@@ -4596,11 +4807,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H111" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="I111" t="n">
-        <v>112.1951219512195</v>
+      <c r="H111">
+        <f>XLOOKUP(C111, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I111">
+        <f>(F111/H111)*100</f>
+        <v/>
       </c>
     </row>
     <row r="112">
@@ -4633,11 +4846,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H112" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="I112" t="n">
-        <v>108.3333333333333</v>
+      <c r="H112">
+        <f>XLOOKUP(C112, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I112">
+        <f>(F112/H112)*100</f>
+        <v/>
       </c>
     </row>
     <row r="113">
@@ -4670,11 +4885,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H113" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="I113" t="n">
-        <v>107.4074074074074</v>
+      <c r="H113">
+        <f>XLOOKUP(C113, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I113">
+        <f>(F113/H113)*100</f>
+        <v/>
       </c>
     </row>
     <row r="114">
@@ -4707,11 +4924,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H114" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="I114" t="n">
-        <v>102.0408163265306</v>
+      <c r="H114">
+        <f>XLOOKUP(C114, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I114">
+        <f>(F114/H114)*100</f>
+        <v/>
       </c>
     </row>
     <row r="115">
@@ -4744,11 +4963,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H115" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="I115" t="n">
-        <v>100</v>
+      <c r="H115">
+        <f>XLOOKUP(C115, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I115">
+        <f>(F115/H115)*100</f>
+        <v/>
       </c>
     </row>
     <row r="116">
@@ -4781,11 +5002,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H116" t="n">
-        <v>446</v>
-      </c>
-      <c r="I116" t="n">
-        <v>100</v>
+      <c r="H116">
+        <f>XLOOKUP(C116, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I116">
+        <f>(F116/H116)*100</f>
+        <v/>
       </c>
     </row>
     <row r="117">
@@ -4818,11 +5041,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H117" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="I117" t="n">
-        <v>100</v>
+      <c r="H117">
+        <f>XLOOKUP(C117, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I117">
+        <f>(F117/H117)*100</f>
+        <v/>
       </c>
     </row>
     <row r="118">
@@ -4855,11 +5080,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H118" t="n">
-        <v>6.12</v>
-      </c>
-      <c r="I118" t="n">
-        <v>100.4901960784314</v>
+      <c r="H118">
+        <f>XLOOKUP(C118, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I118">
+        <f>(F118/H118)*100</f>
+        <v/>
       </c>
     </row>
     <row r="119">
@@ -4892,11 +5119,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H119" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="I119" t="n">
-        <v>100</v>
+      <c r="H119">
+        <f>XLOOKUP(C119, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I119">
+        <f>(F119/H119)*100</f>
+        <v/>
       </c>
     </row>
     <row r="120">
@@ -4929,11 +5158,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H120" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="I120" t="n">
-        <v>100.5747126436782</v>
+      <c r="H120">
+        <f>XLOOKUP(C120, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I120">
+        <f>(F120/H120)*100</f>
+        <v/>
       </c>
     </row>
     <row r="121">
@@ -4966,11 +5197,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H121" t="n">
-        <v>6</v>
-      </c>
-      <c r="I121" t="n">
-        <v>100</v>
+      <c r="H121">
+        <f>XLOOKUP(C121, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I121">
+        <f>(F121/H121)*100</f>
+        <v/>
       </c>
     </row>
     <row r="122">
@@ -5003,11 +5236,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H122" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="I122" t="n">
-        <v>100</v>
+      <c r="H122">
+        <f>XLOOKUP(C122, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I122">
+        <f>(F122/H122)*100</f>
+        <v/>
       </c>
     </row>
     <row r="123">
@@ -5040,11 +5275,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H123" t="n">
-        <v>57</v>
-      </c>
-      <c r="I123" t="n">
-        <v>100</v>
+      <c r="H123">
+        <f>XLOOKUP(C123, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I123">
+        <f>(F123/H123)*100</f>
+        <v/>
       </c>
     </row>
     <row r="124">
@@ -5077,11 +5314,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H124" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="I124" t="n">
-        <v>105.2631578947368</v>
+      <c r="H124">
+        <f>XLOOKUP(C124, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I124">
+        <f>(F124/H124)*100</f>
+        <v/>
       </c>
     </row>
     <row r="125">
@@ -5114,11 +5353,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H125" t="n">
-        <v>44.5</v>
-      </c>
-      <c r="I125" t="n">
-        <v>101.123595505618</v>
+      <c r="H125">
+        <f>XLOOKUP(C125, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I125">
+        <f>(F125/H125)*100</f>
+        <v/>
       </c>
     </row>
     <row r="126">
@@ -5151,11 +5392,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H126" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="I126" t="n">
-        <v>100</v>
+      <c r="H126">
+        <f>XLOOKUP(C126, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I126">
+        <f>(F126/H126)*100</f>
+        <v/>
       </c>
     </row>
     <row r="127">
@@ -5188,11 +5431,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H127" t="n">
-        <v>86.67</v>
-      </c>
-      <c r="I127" t="n">
-        <v>100</v>
+      <c r="H127">
+        <f>XLOOKUP(C127, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I127">
+        <f>(F127/H127)*100</f>
+        <v/>
       </c>
     </row>
     <row r="128">
@@ -5225,11 +5470,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H128" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="I128" t="n">
-        <v>100</v>
+      <c r="H128">
+        <f>XLOOKUP(C128, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I128">
+        <f>(F128/H128)*100</f>
+        <v/>
       </c>
     </row>
     <row r="129">
@@ -5262,11 +5509,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H129" t="n">
-        <v>18.57</v>
-      </c>
-      <c r="I129" t="n">
-        <v>101.2385568120625</v>
+      <c r="H129">
+        <f>XLOOKUP(C129, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I129">
+        <f>(F129/H129)*100</f>
+        <v/>
       </c>
     </row>
     <row r="130">
@@ -5299,11 +5548,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H130" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="I130" t="n">
-        <v>101.1904761904762</v>
+      <c r="H130">
+        <f>XLOOKUP(C130, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I130">
+        <f>(F130/H130)*100</f>
+        <v/>
       </c>
     </row>
     <row r="131">
@@ -5336,11 +5587,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H131" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="I131" t="n">
-        <v>112.1951219512195</v>
+      <c r="H131">
+        <f>XLOOKUP(C131, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I131">
+        <f>(F131/H131)*100</f>
+        <v/>
       </c>
     </row>
     <row r="132">
@@ -5373,11 +5626,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H132" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="I132" t="n">
-        <v>108.3333333333333</v>
+      <c r="H132">
+        <f>XLOOKUP(C132, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I132">
+        <f>(F132/H132)*100</f>
+        <v/>
       </c>
     </row>
     <row r="133">
@@ -5410,11 +5665,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H133" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="I133" t="n">
-        <v>103.7037037037037</v>
+      <c r="H133">
+        <f>XLOOKUP(C133, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I133">
+        <f>(F133/H133)*100</f>
+        <v/>
       </c>
     </row>
     <row r="134">
@@ -5447,11 +5704,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H134" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="I134" t="n">
-        <v>102.0408163265306</v>
+      <c r="H134">
+        <f>XLOOKUP(C134, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I134">
+        <f>(F134/H134)*100</f>
+        <v/>
       </c>
     </row>
     <row r="135">
@@ -5484,11 +5743,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H135" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="I135" t="n">
-        <v>100</v>
+      <c r="H135">
+        <f>XLOOKUP(C135, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I135">
+        <f>(F135/H135)*100</f>
+        <v/>
       </c>
     </row>
     <row r="136">
@@ -5521,11 +5782,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H136" t="n">
-        <v>446</v>
-      </c>
-      <c r="I136" t="n">
-        <v>100</v>
+      <c r="H136">
+        <f>XLOOKUP(C136, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I136">
+        <f>(F136/H136)*100</f>
+        <v/>
       </c>
     </row>
     <row r="137">
@@ -5558,11 +5821,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H137" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="I137" t="n">
-        <v>100</v>
+      <c r="H137">
+        <f>XLOOKUP(C137, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I137">
+        <f>(F137/H137)*100</f>
+        <v/>
       </c>
     </row>
     <row r="138">
@@ -5595,11 +5860,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H138" t="n">
-        <v>6.12</v>
-      </c>
-      <c r="I138" t="n">
-        <v>100.4901960784314</v>
+      <c r="H138">
+        <f>XLOOKUP(C138, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I138">
+        <f>(F138/H138)*100</f>
+        <v/>
       </c>
     </row>
     <row r="139">
@@ -5632,11 +5899,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H139" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="I139" t="n">
-        <v>100</v>
+      <c r="H139">
+        <f>XLOOKUP(C139, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I139">
+        <f>(F139/H139)*100</f>
+        <v/>
       </c>
     </row>
     <row r="140">
@@ -5669,11 +5938,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H140" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="I140" t="n">
-        <v>100.5747126436782</v>
+      <c r="H140">
+        <f>XLOOKUP(C140, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I140">
+        <f>(F140/H140)*100</f>
+        <v/>
       </c>
     </row>
     <row r="141">
@@ -5706,11 +5977,13 @@
           <t>Scraped</t>
         </is>
       </c>
-      <c r="H141" t="n">
-        <v>6</v>
-      </c>
-      <c r="I141" t="n">
-        <v>100</v>
+      <c r="H141">
+        <f>XLOOKUP(C141, $C$2:$C$21, $F$2:$F$21)</f>
+        <v/>
+      </c>
+      <c r="I141">
+        <f>(F141/H141)*100</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -5735,37 +6008,37 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Staples</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Dairy</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Oils</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>Household</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Oils</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Produce</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Snacks</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Staples</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Overall_CPI</t>
+          <t>Overall CPI</t>
         </is>
       </c>
     </row>
@@ -5775,26 +6048,33 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>100</v>
-      </c>
-      <c r="C2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D2" t="n">
-        <v>100</v>
-      </c>
-      <c r="E2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F2" t="n">
-        <v>100</v>
-      </c>
-      <c r="G2" t="n">
-        <v>100</v>
-      </c>
-      <c r="H2" t="n">
-        <v>100</v>
+      <c r="B2">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A2, 'Raw Daily Price Data'!$B:$B, B$1)</f>
+        <v/>
+      </c>
+      <c r="C2">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A2, 'Raw Daily Price Data'!$B:$B, C$1)</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A2, 'Raw Daily Price Data'!$B:$B, D$1)</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A2, 'Raw Daily Price Data'!$B:$B, E$1)</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A2, 'Raw Daily Price Data'!$B:$B, F$1)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A2, 'Raw Daily Price Data'!$B:$B, G$1)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>((B2*0.25) + (C2*0.2) + (D2*0.2) + (E2*0.15) + (F2*0.1) + (G2*0.1)) / (IF(B2&gt;0, 0.25, 0) + IF(C2&gt;0, 0.2, 0) + IF(D2&gt;0, 0.2, 0) + IF(E2&gt;0, 0.15, 0) + IF(F2&gt;0, 0.1, 0) + IF(G2&gt;0, 0.1, 0))</f>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -5803,26 +6083,33 @@
           <t>2026-03-28</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>100.219298245614</v>
-      </c>
-      <c r="C3" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" t="n">
-        <v>100</v>
-      </c>
-      <c r="E3" t="n">
-        <v>103.5343270099368</v>
-      </c>
-      <c r="F3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G3" t="n">
-        <v>100</v>
-      </c>
-      <c r="H3" t="n">
-        <v>100.7507250511102</v>
+      <c r="B3">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A3, 'Raw Daily Price Data'!$B:$B, B$1)</f>
+        <v/>
+      </c>
+      <c r="C3">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A3, 'Raw Daily Price Data'!$B:$B, C$1)</f>
+        <v/>
+      </c>
+      <c r="D3">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A3, 'Raw Daily Price Data'!$B:$B, D$1)</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A3, 'Raw Daily Price Data'!$B:$B, E$1)</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A3, 'Raw Daily Price Data'!$B:$B, F$1)</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A3, 'Raw Daily Price Data'!$B:$B, G$1)</f>
+        <v/>
+      </c>
+      <c r="H3">
+        <f>((B3*0.25) + (C3*0.2) + (D3*0.2) + (E3*0.15) + (F3*0.1) + (G3*0.1)) / (IF(B3&gt;0, 0.25, 0) + IF(C3&gt;0, 0.2, 0) + IF(D3&gt;0, 0.2, 0) + IF(E3&gt;0, 0.15, 0) + IF(F3&gt;0, 0.1, 0) + IF(G3&gt;0, 0.1, 0))</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -5831,26 +6118,33 @@
           <t>2026-03-29</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>101.1580918588606</v>
-      </c>
-      <c r="C4" t="n">
-        <v>100</v>
-      </c>
-      <c r="D4" t="n">
-        <v>100.6192784060312</v>
-      </c>
-      <c r="E4" t="n">
-        <v>110.040466050919</v>
-      </c>
-      <c r="F4" t="n">
-        <v>100</v>
-      </c>
-      <c r="G4" t="n">
-        <v>100.1225490196078</v>
-      </c>
-      <c r="H4" t="n">
-        <v>102.3632405977626</v>
+      <c r="B4">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A4, 'Raw Daily Price Data'!$B:$B, B$1)</f>
+        <v/>
+      </c>
+      <c r="C4">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A4, 'Raw Daily Price Data'!$B:$B, C$1)</f>
+        <v/>
+      </c>
+      <c r="D4">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A4, 'Raw Daily Price Data'!$B:$B, D$1)</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A4, 'Raw Daily Price Data'!$B:$B, E$1)</f>
+        <v/>
+      </c>
+      <c r="F4">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A4, 'Raw Daily Price Data'!$B:$B, F$1)</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A4, 'Raw Daily Price Data'!$B:$B, G$1)</f>
+        <v/>
+      </c>
+      <c r="H4">
+        <f>((B4*0.25) + (C4*0.2) + (D4*0.2) + (E4*0.15) + (F4*0.1) + (G4*0.1)) / (IF(B4&gt;0, 0.25, 0) + IF(C4&gt;0, 0.2, 0) + IF(D4&gt;0, 0.2, 0) + IF(E4&gt;0, 0.15, 0) + IF(F4&gt;0, 0.1, 0) + IF(G4&gt;0, 0.1, 0))</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -5859,26 +6153,33 @@
           <t>2026-03-30</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>101.1580918588606</v>
-      </c>
-      <c r="C5" t="n">
-        <v>100</v>
-      </c>
-      <c r="D5" t="n">
-        <v>101.2145165012693</v>
-      </c>
-      <c r="E5" t="n">
-        <v>112.6488671349299</v>
-      </c>
-      <c r="F5" t="n">
-        <v>100</v>
-      </c>
-      <c r="G5" t="n">
-        <v>100.1225490196078</v>
-      </c>
-      <c r="H5" t="n">
-        <v>102.9742065288505</v>
+      <c r="B5">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A5, 'Raw Daily Price Data'!$B:$B, B$1)</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A5, 'Raw Daily Price Data'!$B:$B, C$1)</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A5, 'Raw Daily Price Data'!$B:$B, D$1)</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A5, 'Raw Daily Price Data'!$B:$B, E$1)</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A5, 'Raw Daily Price Data'!$B:$B, F$1)</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A5, 'Raw Daily Price Data'!$B:$B, G$1)</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>((B5*0.25) + (C5*0.2) + (D5*0.2) + (E5*0.15) + (F5*0.1) + (G5*0.1)) / (IF(B5&gt;0, 0.25, 0) + IF(C5&gt;0, 0.2, 0) + IF(D5&gt;0, 0.2, 0) + IF(E5&gt;0, 0.15, 0) + IF(F5&gt;0, 0.1, 0) + IF(G5&gt;0, 0.1, 0))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -5887,26 +6188,33 @@
           <t>2026-03-31</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>101.1580918588606</v>
-      </c>
-      <c r="C6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" t="n">
-        <v>101.2145165012693</v>
-      </c>
-      <c r="E6" t="n">
-        <v>110.5655338015965</v>
-      </c>
-      <c r="F6" t="n">
-        <v>100</v>
-      </c>
-      <c r="G6" t="n">
-        <v>100.2662271805274</v>
-      </c>
-      <c r="H6" t="n">
-        <v>102.5934594024137</v>
+      <c r="B6">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A6, 'Raw Daily Price Data'!$B:$B, B$1)</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A6, 'Raw Daily Price Data'!$B:$B, C$1)</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A6, 'Raw Daily Price Data'!$B:$B, D$1)</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A6, 'Raw Daily Price Data'!$B:$B, E$1)</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A6, 'Raw Daily Price Data'!$B:$B, F$1)</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A6, 'Raw Daily Price Data'!$B:$B, G$1)</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>((B6*0.25) + (C6*0.2) + (D6*0.2) + (E6*0.15) + (F6*0.1) + (G6*0.1)) / (IF(B6&gt;0, 0.25, 0) + IF(C6&gt;0, 0.2, 0) + IF(D6&gt;0, 0.2, 0) + IF(E6&gt;0, 0.15, 0) + IF(F6&gt;0, 0.1, 0) + IF(G6&gt;0, 0.1, 0))</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -5915,26 +6223,33 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>101.5966883500887</v>
-      </c>
-      <c r="C7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D7" t="n">
-        <v>101.2145165012693</v>
-      </c>
-      <c r="E7" t="n">
-        <v>107.4941697546227</v>
-      </c>
-      <c r="F7" t="n">
-        <v>100</v>
-      </c>
-      <c r="G7" t="n">
-        <v>100.2662271805274</v>
-      </c>
-      <c r="H7" t="n">
-        <v>102.0669058912645</v>
+      <c r="B7">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A7, 'Raw Daily Price Data'!$B:$B, B$1)</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A7, 'Raw Daily Price Data'!$B:$B, C$1)</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A7, 'Raw Daily Price Data'!$B:$B, D$1)</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A7, 'Raw Daily Price Data'!$B:$B, E$1)</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A7, 'Raw Daily Price Data'!$B:$B, F$1)</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A7, 'Raw Daily Price Data'!$B:$B, G$1)</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>((B7*0.25) + (C7*0.2) + (D7*0.2) + (E7*0.15) + (F7*0.1) + (G7*0.1)) / (IF(B7&gt;0, 0.25, 0) + IF(C7&gt;0, 0.2, 0) + IF(D7&gt;0, 0.2, 0) + IF(E7&gt;0, 0.15, 0) + IF(F7&gt;0, 0.1, 0) + IF(G7&gt;0, 0.1, 0))</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -5943,26 +6258,33 @@
           <t>2026-04-02</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>101.5966883500887</v>
-      </c>
-      <c r="C8" t="n">
-        <v>100</v>
-      </c>
-      <c r="D8" t="n">
-        <v>101.2145165012693</v>
-      </c>
-      <c r="E8" t="n">
-        <v>106.5682438286968</v>
-      </c>
-      <c r="F8" t="n">
-        <v>100</v>
-      </c>
-      <c r="G8" t="n">
-        <v>100.2662271805274</v>
-      </c>
-      <c r="H8" t="n">
-        <v>101.8817207060793</v>
+      <c r="B8">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A8, 'Raw Daily Price Data'!$B:$B, B$1)</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A8, 'Raw Daily Price Data'!$B:$B, C$1)</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A8, 'Raw Daily Price Data'!$B:$B, D$1)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A8, 'Raw Daily Price Data'!$B:$B, E$1)</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A8, 'Raw Daily Price Data'!$B:$B, F$1)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>AVERAGEIFS('Raw Daily Price Data'!$I:$I, 'Raw Daily Price Data'!$A:$A, $A8, 'Raw Daily Price Data'!$B:$B, G$1)</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>((B8*0.25) + (C8*0.2) + (D8*0.2) + (E8*0.15) + (F8*0.1) + (G8*0.1)) / (IF(B8&gt;0, 0.25, 0) + IF(C8&gt;0, 0.2, 0) + IF(D8&gt;0, 0.2, 0) + IF(E8&gt;0, 0.15, 0) + IF(F8&gt;0, 0.1, 0) + IF(G8&gt;0, 0.1, 0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>